<commit_message>
feat: implementado os testes para regras de negocio 7
</commit_message>
<xml_diff>
--- a/data/samples/inspecao_lotes_dia_teste.xlsx
+++ b/data/samples/inspecao_lotes_dia_teste.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,7 +8,7 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Inspecao_14_06_2026" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Inspecao" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Base_Referencia" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Formulario_Analise" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
@@ -651,132 +651,136 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -860,34 +864,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1033,757 +1037,757 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="42"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="4"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="5"/>
+      <c r="H5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="6"/>
+      <c r="H6" s="7"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="E8" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="F8" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="6"/>
+      <c r="H10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H11" s="5"/>
+      <c r="H11" s="6"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="6" t="s">
+      <c r="F12" s="10"/>
+      <c r="G12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="H12" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H13" s="5"/>
+      <c r="H13" s="6"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+      <c r="A14" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H14" s="4"/>
+      <c r="H14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H15" s="6"/>
+      <c r="H15" s="7"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H16" s="4"/>
+      <c r="H16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G17" s="5" t="s">
+      <c r="G17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="H18" s="6"/>
+      <c r="H18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G19" s="5" t="s">
+      <c r="G19" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H20" s="4"/>
+      <c r="H20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="E21" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H21" s="6" t="s">
+      <c r="H21" s="7" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="A22" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H22" s="4"/>
+      <c r="H22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G23" s="5" t="s">
+      <c r="G23" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H23" s="5"/>
+      <c r="H23" s="6"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="6"/>
+      <c r="H24" s="7"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="G25" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H25" s="5"/>
+      <c r="H25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D26" s="4" t="s">
+      <c r="D26" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E26" s="4" t="s">
+      <c r="E26" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="4" t="s">
+      <c r="F26" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G26" s="4" t="s">
+      <c r="G26" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H26" s="4"/>
+      <c r="H26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="9"/>
-      <c r="B27" s="6" t="s">
+      <c r="A27" s="10"/>
+      <c r="B27" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="G27" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="H27" s="6"/>
+      <c r="H27" s="7"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="5" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="11" t="s">
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="13"/>
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="14" t="s">
+      <c r="B32" s="14"/>
+      <c r="C32" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="14"/>
-      <c r="E32" s="14"/>
-      <c r="F32" s="14"/>
-      <c r="G32" s="14"/>
-      <c r="H32" s="14"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="16" t="s">
         <v>75</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="14" t="s">
+      <c r="B33" s="16"/>
+      <c r="C33" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="B34" s="16"/>
-      <c r="C34" s="14" t="s">
+      <c r="B34" s="17"/>
+      <c r="C34" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
+      <c r="A35" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="14" t="s">
+      <c r="B35" s="18"/>
+      <c r="C35" s="15" t="s">
         <v>79</v>
       </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -1817,365 +1821,365 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C5" s="19" t="s">
+      <c r="C5" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="B7" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="19" t="s">
+      <c r="C7" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="B9" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="22" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="D10" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="21" t="s">
+      <c r="A12" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="19" t="s">
+      <c r="C13" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="21" t="s">
+      <c r="A14" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="22" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="22" t="s">
+      <c r="D14" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
+      <c r="A15" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="22" t="s">
         <v>94</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="19" t="s">
+      <c r="A17" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="19" t="s">
+      <c r="C17" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="22" t="s">
         <v>88</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="B19" s="19" t="s">
+      <c r="B19" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="19" t="s">
+      <c r="C19" s="20" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="D20" s="22" t="s">
+      <c r="D20" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="19" t="s">
+      <c r="C21" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="22" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19" t="s">
+      <c r="A23" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="20" t="s">
         <v>87</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="D24" s="22" t="s">
+      <c r="D24" s="23" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="19" t="s">
+      <c r="A25" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="C25" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="23" t="s">
+      <c r="A27" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
+      <c r="B27" s="24"/>
+      <c r="C27" s="24"/>
+      <c r="D27" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2198,395 +2202,395 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F38"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
     </row>
     <row r="2" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
+      <c r="F2" s="26"/>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="26" t="n">
+      <c r="A4" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="n">
+      <c r="A5" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="28"/>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
     </row>
     <row r="6" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="26" t="n">
+      <c r="A6" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="27" t="n">
+      <c r="A7" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="28"/>
-      <c r="C7" s="28"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="29"/>
+      <c r="D7" s="29"/>
+      <c r="E7" s="29"/>
+      <c r="F7" s="29"/>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="n">
+      <c r="A8" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="27" t="n">
+      <c r="A9" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
     </row>
     <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="26" t="n">
+      <c r="A10" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="27" t="n">
+      <c r="A11" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="28"/>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="26" t="n">
+      <c r="A12" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="27" t="n">
+      <c r="A13" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="28"/>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="28"/>
-      <c r="F13" s="28"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="26" t="n">
+      <c r="A14" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="27" t="n">
+      <c r="A15" s="28" t="n">
         <v>12</v>
       </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="29"/>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="26" t="n">
+      <c r="A16" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="27" t="n">
+      <c r="A17" s="28" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28"/>
-      <c r="F17" s="28"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
     </row>
     <row r="18" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="26" t="n">
+      <c r="A18" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="5"/>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-      <c r="E18" s="5"/>
-      <c r="F18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="27" t="n">
+      <c r="A19" s="28" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
     </row>
     <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="26" t="n">
+      <c r="A20" s="27" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="27" t="n">
+      <c r="A21" s="28" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="28"/>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-      <c r="F21" s="28"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
     </row>
     <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="26" t="n">
+      <c r="A22" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-      <c r="E22" s="5"/>
-      <c r="F22" s="5"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="27" t="n">
+      <c r="A23" s="28" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="29"/>
+      <c r="F23" s="29"/>
     </row>
     <row r="24" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="26" t="n">
+      <c r="A24" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="27" t="n">
+      <c r="A25" s="28" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="28"/>
-      <c r="C25" s="28"/>
-      <c r="D25" s="28"/>
-      <c r="E25" s="28"/>
-      <c r="F25" s="28"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="29"/>
+      <c r="F25" s="29"/>
     </row>
     <row r="26" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="26" t="n">
+      <c r="A26" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
     </row>
     <row r="27" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="27" t="n">
+      <c r="A27" s="28" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="28"/>
-      <c r="C27" s="28"/>
-      <c r="D27" s="28"/>
-      <c r="E27" s="28"/>
-      <c r="F27" s="28"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
     </row>
     <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="n">
+      <c r="A28" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="B30" s="12"/>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
     </row>
     <row r="31" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="30"/>
-      <c r="C31" s="30"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
+      <c r="B31" s="31"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
     </row>
     <row r="32" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="30" t="s">
+      <c r="A32" s="31" t="s">
         <v>105</v>
       </c>
-      <c r="B32" s="30"/>
-      <c r="C32" s="30"/>
-      <c r="D32" s="31"/>
-      <c r="E32" s="31"/>
-      <c r="F32" s="31"/>
+      <c r="B32" s="31"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="32"/>
+      <c r="F32" s="32"/>
     </row>
     <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="30" t="s">
+      <c r="A33" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="B33" s="30"/>
-      <c r="C33" s="30"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="31"/>
+      <c r="B33" s="31"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="32"/>
+      <c r="E33" s="32"/>
+      <c r="F33" s="32"/>
     </row>
     <row r="34" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="30" t="s">
+      <c r="A34" s="31" t="s">
         <v>107</v>
       </c>
-      <c r="B34" s="30"/>
-      <c r="C34" s="30"/>
-      <c r="D34" s="31"/>
-      <c r="E34" s="31"/>
-      <c r="F34" s="31"/>
+      <c r="B34" s="31"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="32"/>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
     </row>
     <row r="35" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="30" t="s">
+      <c r="A35" s="31" t="s">
         <v>108</v>
       </c>
-      <c r="B35" s="30"/>
-      <c r="C35" s="30"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
     </row>
     <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="30" t="s">
+      <c r="A36" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="B36" s="30"/>
-      <c r="C36" s="30"/>
-      <c r="D36" s="31"/>
-      <c r="E36" s="31"/>
-      <c r="F36" s="31"/>
+      <c r="B36" s="31"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
     </row>
     <row r="37" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30" t="s">
+      <c r="A37" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="B37" s="30"/>
-      <c r="C37" s="30"/>
-      <c r="D37" s="31"/>
-      <c r="E37" s="31"/>
-      <c r="F37" s="31"/>
+      <c r="B37" s="31"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="32"/>
+      <c r="E37" s="32"/>
+      <c r="F37" s="32"/>
     </row>
     <row r="38" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="30" t="s">
+      <c r="A38" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
-      <c r="D38" s="31"/>
-      <c r="E38" s="31"/>
-      <c r="F38" s="31"/>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="32"/>
+      <c r="F38" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>